<commit_message>
fix: universal Excel upload support for Benefits and Tax tabs across all formats, versions, and platforms
</commit_message>
<xml_diff>
--- a/data/tax.xlsx
+++ b/data/tax.xlsx
@@ -1,47 +1,47 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
+    <sheet name="MacroFirstSheet" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
-  <si>
-    <t>Batch Name/Job Name</t>
-  </si>
-  <si>
-    <t>Schedule Name/ Job Group Name</t>
-  </si>
-  <si>
-    <t>Batch Arguments/JVM Arguments</t>
-  </si>
-  <si>
-    <t>TestTaxSheet1Batch</t>
-  </si>
-  <si>
-    <t>benefits_weekly_monday_515pm</t>
-  </si>
-  <si>
-    <t>-Xmx1024m</t>
-  </si>
-</sst>
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <numFmts count="1">
+    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+  </numFmts>
+  <fonts count="1">
     <font>
+      <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -65,21 +65,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
 </styleSheet>
 </file>
 
@@ -404,34 +396,40 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D2"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Job Name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>JVM Arguments</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Job Group Name</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Trigger Needed</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" t="s">
-        <v>5</v>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>MacroBatchJob</v>
+      </c>
+      <c r="B2" t="str">
+        <v>MODE=BATCH</v>
+      </c>
+      <c r="C2" t="str">
+        <v>benefits_weekly_monday_515pm</v>
+      </c>
+      <c r="D2" t="str">
+        <v>N</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>